<commit_message>
Update my appointment TestCase
</commit_message>
<xml_diff>
--- a/TestCases/My_Appointment_TestCase.xlsx
+++ b/TestCases/My_Appointment_TestCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BA4AD8A-4510-4DEA-9378-5E96487C88BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB240A20-BFA2-4FCD-BDE6-9C544EFE289F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -194,10 +194,10 @@
 Không phát sinh thêm bản ghi lịch hẹn trùng.</t>
   </si>
   <si>
-    <t>TCMyAppointment4_1, TCMyAppointment4_2, TCMyAppointment4_2, TCMyAppointment4_4</t>
+    <t>TCMyAppointment4_1, TCMyAppointment4_2, TCMyAppointment4_3, TCMyAppointment4_4</t>
   </si>
   <si>
-    <t>Lịch hẹn sau khi Admin xác nhận được hiển thị đúng phía Doctor và Doctor có thể mở chức năng khám cho lịch hẹn tương ứng.</t>
+    <t>Lịch hẹn được cập nhật đúng xuyên suốt từ “Chờ xác nhận” -&gt; “Đã xác nhận” -&gt; “Đã hoàn thành” sau khi Doctor hoàn tất khám.</t>
   </si>
   <si>
     <t>4. Kiểm tra khung giờ được giải phóng sau khi lịch hẹn bị hủy</t>
@@ -224,7 +224,7 @@
 Lịch mới có ID khác và trạng thái “Chờ xác nhận”.</t>
   </si>
   <si>
-    <t>TCMyAppointment5_1, TCMyAppointment5_2, TCMyAppointment5_2</t>
+    <t>TCMyAppointment5_1, TCMyAppointment5_2, TCMyAppointment5_3</t>
   </si>
   <si>
     <t>Lịch hẹn đã hủy không còn chiếm khung giờ, hệ thống cho phép tạo lịch mới tại cùng ngày giờ với trạng thái “Chờ xác nhận”.</t>
@@ -29368,21 +29368,21 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A19:J19"/>
     <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D18:F18"/>
     <mergeCell ref="D9:F10"/>
-    <mergeCell ref="B11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A19:J19"/>
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="I9:I10"/>
     <mergeCell ref="J9:J10"/>
+    <mergeCell ref="B11:J11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A14:J14"/>
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="B1:D2"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B4:D4"/>

</xml_diff>